<commit_message>
Working code for METALS demo
</commit_message>
<xml_diff>
--- a/DataVaryingTemperature/3Materials.xlsx
+++ b/DataVaryingTemperature/3Materials.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Personal\suresh\Software\Github\ERSL-Private\METALS\DataVaryingTemperature\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39569C5F-9010-49BA-B445-D38885D08DB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7457294-CBC0-4DAD-8ECC-276FD143515C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1968" yWindow="3360" windowWidth="20604" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1392" yWindow="1536" windowWidth="20604" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -166,7 +166,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -191,9 +191,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="14"/>
-      <color rgb="FF0070C0"/>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -210,6 +208,14 @@
       <b/>
       <sz val="14"/>
       <color theme="5" tint="-0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF0070C0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -268,7 +274,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -318,13 +324,19 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="11" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -733,7 +745,7 @@
       </c>
     </row>
     <row r="3" spans="1:22" ht="18" x14ac:dyDescent="0.3">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="21" t="s">
         <v>34</v>
       </c>
       <c r="B3" s="7">
@@ -746,29 +758,31 @@
         <v>92976880986.810806</v>
       </c>
       <c r="E3" s="12">
-        <f t="shared" ref="E3" si="0">D3*EXP(-2000/Q3)</f>
+        <f t="shared" ref="E3:E5" si="0">D3*EXP(-2000/Q3)</f>
         <v>306684777.10425931</v>
       </c>
       <c r="F3" s="12">
-        <f t="shared" ref="F3" si="1">0.1*D3*EXP(-3000/Q3)</f>
+        <f t="shared" ref="F3:F5" si="1">0.1*D3*EXP(-3000/Q3)</f>
         <v>1761371.0038603023</v>
       </c>
       <c r="G3" s="12">
-        <v>0.99992423656867901</v>
+        <f t="shared" ref="G3:G5" si="2">0.1*F3</f>
+        <v>176137.10038603024</v>
       </c>
       <c r="H3" s="12">
         <v>413532439.30818099</v>
       </c>
       <c r="I3" s="12">
-        <f t="shared" ref="I3" si="2">0.1*H3*EXP(-2000/Q3)</f>
+        <f t="shared" ref="I3:I5" si="3">0.1*H3*EXP(-2000/Q3)</f>
         <v>136403.9131325568</v>
       </c>
       <c r="J3" s="12">
-        <f t="shared" ref="J3" si="3">0.1*H3*EXP(-3000/Q3)</f>
+        <f t="shared" ref="J3:J5" si="4">0.1*H3*EXP(-3000/Q3)</f>
         <v>7834.0340095552874</v>
       </c>
-      <c r="K3" s="12">
-        <v>1.0004243155682</v>
+      <c r="K3" s="17">
+        <f t="shared" ref="K3:K5" si="5">0.1*J3</f>
+        <v>783.40340095552881</v>
       </c>
       <c r="L3" s="8">
         <v>155</v>
@@ -785,7 +799,7 @@
       <c r="P3" s="15">
         <v>0.15</v>
       </c>
-      <c r="Q3" s="12">
+      <c r="Q3" s="18">
         <v>350</v>
       </c>
       <c r="R3" s="8">
@@ -793,7 +807,7 @@
       </c>
     </row>
     <row r="4" spans="1:22" ht="18" x14ac:dyDescent="0.3">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="19" t="s">
         <v>35</v>
       </c>
       <c r="B4" s="7">
@@ -806,25 +820,31 @@
         <v>54070808940.932602</v>
       </c>
       <c r="E4" s="12">
-        <v>53063644666.036102</v>
+        <f t="shared" si="0"/>
+        <v>8048876846.430934</v>
       </c>
       <c r="F4" s="12">
-        <v>171529075344.30801</v>
+        <f t="shared" si="1"/>
+        <v>310542818.33966625</v>
       </c>
       <c r="G4" s="12">
-        <v>1.0006921851331401</v>
+        <f t="shared" si="2"/>
+        <v>31054281.833966628</v>
       </c>
       <c r="H4" s="12">
         <v>384064916.71307498</v>
       </c>
       <c r="I4" s="12">
-        <v>67336407.728308499</v>
+        <f t="shared" si="3"/>
+        <v>5717116.640580033</v>
       </c>
       <c r="J4" s="12">
-        <v>9802478271.9358501</v>
-      </c>
-      <c r="K4" s="12">
-        <v>0.99970767300819297</v>
+        <f t="shared" si="4"/>
+        <v>2205785.4135631202</v>
+      </c>
+      <c r="K4" s="17">
+        <f t="shared" si="5"/>
+        <v>220578.54135631202</v>
       </c>
       <c r="L4" s="8">
         <v>15</v>
@@ -841,7 +861,7 @@
       <c r="P4" s="15">
         <v>0.46</v>
       </c>
-      <c r="Q4" s="12">
+      <c r="Q4" s="18">
         <v>1050</v>
       </c>
       <c r="R4" s="8">
@@ -851,7 +871,7 @@
       <c r="V4" s="5"/>
     </row>
     <row r="5" spans="1:22" ht="18" x14ac:dyDescent="0.3">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="20" t="s">
         <v>36</v>
       </c>
       <c r="B5" s="7">
@@ -864,25 +884,31 @@
         <v>117108650073.651</v>
       </c>
       <c r="E5" s="12">
-        <v>44884386172.699799</v>
+        <f t="shared" si="0"/>
+        <v>22118966880.153912</v>
       </c>
       <c r="F5" s="12">
-        <v>175213569928.29001</v>
+        <f t="shared" si="1"/>
+        <v>961286338.01422894</v>
       </c>
       <c r="G5" s="12">
-        <v>1.0007894571356</v>
+        <f t="shared" si="2"/>
+        <v>96128633.801422894</v>
       </c>
       <c r="H5" s="12">
         <v>425435242.49228698</v>
       </c>
       <c r="I5" s="12">
-        <v>77030174.758169293</v>
+        <f t="shared" si="3"/>
+        <v>8035433.789407501</v>
       </c>
       <c r="J5" s="12">
-        <v>751102621.40532196</v>
-      </c>
-      <c r="K5" s="12">
-        <v>0.99976714584067305</v>
+        <f t="shared" si="4"/>
+        <v>3492185.1294537433</v>
+      </c>
+      <c r="K5" s="17">
+        <f t="shared" si="5"/>
+        <v>349218.51294537436</v>
       </c>
       <c r="L5" s="8">
         <v>17</v>
@@ -899,7 +925,7 @@
       <c r="P5" s="15">
         <v>1E-3</v>
       </c>
-      <c r="Q5" s="12">
+      <c r="Q5" s="18">
         <v>1200</v>
       </c>
       <c r="R5" s="8">

</xml_diff>

<commit_message>
Removed torch from sensitivities files
</commit_message>
<xml_diff>
--- a/DataVaryingTemperature/3Materials.xlsx
+++ b/DataVaryingTemperature/3Materials.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Personal\suresh\Software\Github\ERSL-Private\METALS\DataVaryingTemperature\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7457294-CBC0-4DAD-8ECC-276FD143515C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFEA1425-D373-4DDF-86E5-DB7EC2F70FF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1392" yWindow="1536" windowWidth="20604" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1500" yWindow="1500" windowWidth="20604" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="39">
   <si>
     <t>Attribute</t>
   </si>
@@ -619,87 +619,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V11"/>
+  <dimension ref="A1:W11"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.6640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="14" style="1" customWidth="1"/>
-    <col min="3" max="3" width="12.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="6" width="9.33203125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="12.44140625" style="1" customWidth="1"/>
-    <col min="8" max="10" width="11.6640625" style="1" customWidth="1"/>
-    <col min="11" max="14" width="10.44140625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="10" style="1" customWidth="1"/>
-    <col min="16" max="16" width="13.6640625" style="1" customWidth="1"/>
-    <col min="17" max="17" width="16.5546875" style="1" customWidth="1"/>
-    <col min="18" max="704" width="20.5546875" style="1" customWidth="1"/>
-    <col min="705" max="16384" width="9.109375" style="1"/>
+    <col min="2" max="2" width="10" style="1" customWidth="1"/>
+    <col min="3" max="3" width="14" style="1" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="9.33203125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="12.44140625" style="1" customWidth="1"/>
+    <col min="9" max="11" width="11.6640625" style="1" customWidth="1"/>
+    <col min="12" max="15" width="10.44140625" style="1" customWidth="1"/>
+    <col min="16" max="16" width="10" style="1" customWidth="1"/>
+    <col min="17" max="17" width="13.6640625" style="1" customWidth="1"/>
+    <col min="18" max="18" width="16.5546875" style="1" customWidth="1"/>
+    <col min="19" max="705" width="20.5546875" style="1" customWidth="1"/>
+    <col min="706" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:23" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.3">
       <c r="A1" s="3"/>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="D1" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="E1" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="F1" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="G1" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="H1" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="I1" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="J1" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="K1" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="K1" s="10" t="s">
+      <c r="L1" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="M1" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="N1" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="O1" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="P1" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="P1" s="14" t="s">
+      <c r="Q1" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="R1" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="R1" s="6" t="s">
+      <c r="S1" s="6" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A2" s="4"/>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="4"/>
+      <c r="C2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="D2" s="15" t="s">
         <v>27</v>
-      </c>
-      <c r="D2" s="11" t="s">
-        <v>12</v>
       </c>
       <c r="E2" s="11" t="s">
         <v>12</v>
@@ -722,8 +724,8 @@
       <c r="K2" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="L2" s="7" t="s">
-        <v>21</v>
+      <c r="L2" s="11" t="s">
+        <v>12</v>
       </c>
       <c r="M2" s="7" t="s">
         <v>21</v>
@@ -734,58 +736,61 @@
       <c r="O2" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="P2" s="15" t="s">
+      <c r="P2" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q2" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="Q2" s="7" t="s">
+      <c r="R2" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="R2" s="7" t="s">
+      <c r="S2" s="7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:22" ht="18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:23" ht="18" x14ac:dyDescent="0.3">
       <c r="A3" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="21">
+        <v>6</v>
+      </c>
+      <c r="C3" s="7">
         <v>2810</v>
       </c>
-      <c r="C3" s="15">
+      <c r="D3" s="15">
         <v>1.28</v>
       </c>
-      <c r="D3" s="12">
+      <c r="E3" s="12">
         <v>92976880986.810806</v>
       </c>
-      <c r="E3" s="12">
-        <f t="shared" ref="E3:E5" si="0">D3*EXP(-2000/Q3)</f>
+      <c r="F3" s="12">
+        <f t="shared" ref="F3:F5" si="0">E3*EXP(-2000/R3)</f>
         <v>306684777.10425931</v>
       </c>
-      <c r="F3" s="12">
-        <f t="shared" ref="F3:F5" si="1">0.1*D3*EXP(-3000/Q3)</f>
+      <c r="G3" s="12">
+        <f t="shared" ref="G3:G5" si="1">0.1*E3*EXP(-3000/R3)</f>
         <v>1761371.0038603023</v>
       </c>
-      <c r="G3" s="12">
-        <f t="shared" ref="G3:G5" si="2">0.1*F3</f>
+      <c r="H3" s="12">
+        <f t="shared" ref="H3:H5" si="2">0.1*G3</f>
         <v>176137.10038603024</v>
       </c>
-      <c r="H3" s="12">
+      <c r="I3" s="12">
         <v>413532439.30818099</v>
       </c>
-      <c r="I3" s="12">
-        <f t="shared" ref="I3:I5" si="3">0.1*H3*EXP(-2000/Q3)</f>
+      <c r="J3" s="12">
+        <f t="shared" ref="J3:J5" si="3">0.1*I3*EXP(-2000/R3)</f>
         <v>136403.9131325568</v>
       </c>
-      <c r="J3" s="12">
-        <f t="shared" ref="J3:J5" si="4">0.1*H3*EXP(-3000/Q3)</f>
+      <c r="K3" s="12">
+        <f t="shared" ref="K3:K5" si="4">0.1*I3*EXP(-3000/R3)</f>
         <v>7834.0340095552874</v>
       </c>
-      <c r="K3" s="17">
-        <f t="shared" ref="K3:K5" si="5">0.1*J3</f>
+      <c r="L3" s="17">
+        <f t="shared" ref="L3:L5" si="5">0.1*K3</f>
         <v>783.40340095552881</v>
-      </c>
-      <c r="L3" s="8">
-        <v>155</v>
       </c>
       <c r="M3" s="8">
         <v>155</v>
@@ -796,150 +801,159 @@
       <c r="O3" s="8">
         <v>155</v>
       </c>
-      <c r="P3" s="15">
+      <c r="P3" s="8">
+        <v>155</v>
+      </c>
+      <c r="Q3" s="15">
         <v>0.15</v>
       </c>
-      <c r="Q3" s="18">
+      <c r="R3" s="18">
         <v>350</v>
       </c>
-      <c r="R3" s="8">
+      <c r="S3" s="8">
         <v>150000000</v>
       </c>
     </row>
-    <row r="4" spans="1:22" ht="18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:23" ht="18" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B4" s="19">
+        <v>3</v>
+      </c>
+      <c r="C4" s="7">
         <v>8000</v>
       </c>
-      <c r="C4" s="15">
+      <c r="D4" s="15">
         <v>1.75</v>
       </c>
-      <c r="D4" s="12">
+      <c r="E4" s="12">
         <v>54070808940.932602</v>
       </c>
-      <c r="E4" s="12">
+      <c r="F4" s="12">
         <f t="shared" si="0"/>
         <v>8048876846.430934</v>
       </c>
-      <c r="F4" s="12">
+      <c r="G4" s="12">
         <f t="shared" si="1"/>
         <v>310542818.33966625</v>
       </c>
-      <c r="G4" s="12">
+      <c r="H4" s="12">
         <f t="shared" si="2"/>
         <v>31054281.833966628</v>
       </c>
-      <c r="H4" s="12">
+      <c r="I4" s="12">
         <v>384064916.71307498</v>
       </c>
-      <c r="I4" s="12">
+      <c r="J4" s="12">
         <f t="shared" si="3"/>
         <v>5717116.640580033</v>
       </c>
-      <c r="J4" s="12">
+      <c r="K4" s="12">
         <f t="shared" si="4"/>
         <v>2205785.4135631202</v>
       </c>
-      <c r="K4" s="17">
+      <c r="L4" s="17">
         <f t="shared" si="5"/>
         <v>220578.54135631202</v>
       </c>
-      <c r="L4" s="8">
+      <c r="M4" s="8">
         <v>15</v>
       </c>
-      <c r="M4" s="8">
+      <c r="N4" s="8">
         <v>20</v>
       </c>
-      <c r="N4" s="8">
+      <c r="O4" s="8">
         <v>29.6</v>
       </c>
-      <c r="O4" s="7">
+      <c r="P4" s="7">
         <v>26</v>
       </c>
-      <c r="P4" s="15">
+      <c r="Q4" s="15">
         <v>0.46</v>
       </c>
-      <c r="Q4" s="18">
+      <c r="R4" s="18">
         <v>1050</v>
       </c>
-      <c r="R4" s="8">
+      <c r="S4" s="8">
         <v>229000000</v>
       </c>
-      <c r="T4" s="5"/>
-      <c r="V4" s="5"/>
-    </row>
-    <row r="5" spans="1:22" ht="18" x14ac:dyDescent="0.3">
+      <c r="U4" s="5"/>
+      <c r="W4" s="5"/>
+    </row>
+    <row r="5" spans="1:23" ht="18" x14ac:dyDescent="0.3">
       <c r="A5" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="20">
+        <v>11</v>
+      </c>
+      <c r="C5" s="7">
         <v>4410</v>
       </c>
-      <c r="C5" s="15">
+      <c r="D5" s="15">
         <v>1.75</v>
       </c>
-      <c r="D5" s="12">
+      <c r="E5" s="12">
         <v>117108650073.651</v>
       </c>
-      <c r="E5" s="12">
+      <c r="F5" s="12">
         <f t="shared" si="0"/>
         <v>22118966880.153912</v>
       </c>
-      <c r="F5" s="12">
+      <c r="G5" s="12">
         <f t="shared" si="1"/>
         <v>961286338.01422894</v>
       </c>
-      <c r="G5" s="12">
+      <c r="H5" s="12">
         <f t="shared" si="2"/>
         <v>96128633.801422894</v>
       </c>
-      <c r="H5" s="12">
+      <c r="I5" s="12">
         <v>425435242.49228698</v>
       </c>
-      <c r="I5" s="12">
+      <c r="J5" s="12">
         <f t="shared" si="3"/>
         <v>8035433.789407501</v>
       </c>
-      <c r="J5" s="12">
+      <c r="K5" s="12">
         <f t="shared" si="4"/>
         <v>3492185.1294537433</v>
       </c>
-      <c r="K5" s="17">
+      <c r="L5" s="17">
         <f t="shared" si="5"/>
         <v>349218.51294537436</v>
       </c>
-      <c r="L5" s="8">
-        <v>17</v>
-      </c>
       <c r="M5" s="8">
         <v>17</v>
       </c>
       <c r="N5" s="8">
         <v>17</v>
       </c>
-      <c r="O5" s="7">
+      <c r="O5" s="8">
         <v>17</v>
       </c>
-      <c r="P5" s="15">
+      <c r="P5" s="7">
+        <v>17</v>
+      </c>
+      <c r="Q5" s="15">
         <v>1E-3</v>
       </c>
-      <c r="Q5" s="18">
+      <c r="R5" s="18">
         <v>1200</v>
       </c>
-      <c r="R5" s="8">
+      <c r="S5" s="8">
         <v>245000000</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="B9" s="13"/>
-    </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="B10" s="9"/>
-    </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="B11" s="16"/>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="C9" s="13"/>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="C10" s="9"/>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="C11" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
MMTO cleaned up to be consistent with PyTO changes.
</commit_message>
<xml_diff>
--- a/DataVaryingTemperature/3Materials.xlsx
+++ b/DataVaryingTemperature/3Materials.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Personal\suresh\Software\Github\ERSL-Private\METALS\DataVaryingTemperature\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFEA1425-D373-4DDF-86E5-DB7EC2F70FF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD70C200-4621-4EF8-A44B-9EA56DF1F11A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1500" yWindow="1500" windowWidth="20604" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="40">
   <si>
     <t>Attribute</t>
   </si>
@@ -160,6 +160,9 @@
   </si>
   <si>
     <t>Fatigue_Limit</t>
+  </si>
+  <si>
+    <t>$/kg</t>
   </si>
 </sst>
 </file>
@@ -696,7 +699,9 @@
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A2" s="4"/>
-      <c r="B2" s="4"/>
+      <c r="B2" s="4" t="s">
+        <v>39</v>
+      </c>
       <c r="C2" s="7" t="s">
         <v>7</v>
       </c>

</xml_diff>